<commit_message>
Actualización SNIES y dashboard: 2026-07-28
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V170"/>
+  <dimension ref="A1:V173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17068,10 +17068,8 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>1704</t>
-        </is>
+      <c r="A170" t="n">
+        <v>1704</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -17123,7 +17121,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N170" s="2" t="n">
+      <c r="N170" s="1" t="n">
         <v>45189</v>
       </c>
       <c r="O170" t="inlineStr">
@@ -17158,6 +17156,300 @@
         </is>
       </c>
       <c r="V170" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>1723</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD PONTIFICIA BOLIVARIANA</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Bucaramanga</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>52363</v>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>COMUNICACION SOCIAL Y PERIODISMO</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>144</v>
+      </c>
+      <c r="J171" t="n">
+        <v>8</v>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L171" t="n">
+        <v>10034460</v>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N171" s="2" t="n">
+        <v>45365</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>Ciencias Sociales, Periodismo e Información</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>Periodismo e información</t>
+        </is>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>Periodismo, comunicación y reportajes</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>Comunicación social, periodismo y afines</t>
+        </is>
+      </c>
+      <c r="S171" t="inlineStr"/>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>Humanidades y Cs. Sociales</t>
+        </is>
+      </c>
+      <c r="V171" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>1812</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DE MEDELLIN</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>105468</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>DISEÑO Y GESTIÓN DEL PRODUCTO</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>142</v>
+      </c>
+      <c r="J172" t="n">
+        <v>8</v>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L172" t="n">
+        <v>8587000</v>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N172" s="2" t="n">
+        <v>45104</v>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>Arte y Humanidades</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>Diseño industrial, de moda e interiores</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr"/>
+      <c r="T172" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>Escuela de Arquitectura, Urbanismo y Diseño</t>
+        </is>
+      </c>
+      <c r="V172" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>4721</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSITARIA HORIZONTE</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>107213</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>DERECHO</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>164</v>
+      </c>
+      <c r="J173" t="n">
+        <v>10</v>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L173" t="n">
+        <v>5826000</v>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N173" s="2" t="n">
+        <v>43307</v>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>Derecho</t>
+        </is>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>Derecho</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>Derecho y afines</t>
+        </is>
+      </c>
+      <c r="S173" t="inlineStr"/>
+      <c r="T173" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>Derecho, C. Política y Rel. Internacionales</t>
+        </is>
+      </c>
+      <c r="V173" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-08-04
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V173"/>
+  <dimension ref="A1:V174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17162,10 +17162,8 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>1723</t>
-        </is>
+      <c r="A171" t="n">
+        <v>1723</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -17219,7 +17217,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N171" s="2" t="n">
+      <c r="N171" s="1" t="n">
         <v>45365</v>
       </c>
       <c r="O171" t="inlineStr">
@@ -17260,10 +17258,8 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>1812</t>
-        </is>
+      <c r="A172" t="n">
+        <v>1812</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -17317,7 +17313,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N172" s="2" t="n">
+      <c r="N172" s="1" t="n">
         <v>45104</v>
       </c>
       <c r="O172" t="inlineStr">
@@ -17358,10 +17354,8 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>4721</t>
-        </is>
+      <c r="A173" t="n">
+        <v>4721</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -17415,7 +17409,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N173" s="2" t="n">
+      <c r="N173" s="1" t="n">
         <v>43307</v>
       </c>
       <c r="O173" t="inlineStr">
@@ -17450,6 +17444,102 @@
         </is>
       </c>
       <c r="V173" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2805</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD SIMÓN BOLÍVAR</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Norte de Santander</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>San José de Cúcuta</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>108783</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>MATEMATICAS Y CIENCIAS DE LA COMPUTACION</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>150</v>
+      </c>
+      <c r="J174" t="n">
+        <v>9</v>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N174" s="2" t="n">
+        <v>43826</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>Ciencias Naturales, Matemáticas y Estadística</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>Matemáticas y estadística</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>Matemáticas, estadística y afines</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr"/>
+      <c r="T174" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>Ciencias Básicas</t>
+        </is>
+      </c>
+      <c r="V174" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-08-11
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V174"/>
+  <dimension ref="A1:V178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17450,10 +17450,8 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>2805</t>
-        </is>
+      <c r="A174" t="n">
+        <v>2805</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -17505,7 +17503,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N174" s="2" t="n">
+      <c r="N174" s="1" t="n">
         <v>43826</v>
       </c>
       <c r="O174" t="inlineStr">
@@ -17540,6 +17538,394 @@
         </is>
       </c>
       <c r="V174" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>1111</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD TECNOLOGICA DE PEREIRA - UTP</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Pueblo Rico</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>117436</v>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>LICENCIATURA EN LITERATURA Y LENGUA CASTELLANA</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Híbrida (Presencial-Virtual)</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>159</v>
+      </c>
+      <c r="J175" t="n">
+        <v>10</v>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr"/>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>Por cohorte</t>
+        </is>
+      </c>
+      <c r="N175" s="2" t="n">
+        <v>43704</v>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>Ciencias de la educación</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="S175" t="inlineStr"/>
+      <c r="T175" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>Instituto de Estudios en Educación</t>
+        </is>
+      </c>
+      <c r="V175" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>1709</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD CENTRAL</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>15706</v>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>ECONOMIA</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>143</v>
+      </c>
+      <c r="J176" t="n">
+        <v>9</v>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N176" s="2" t="n">
+        <v>45906</v>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>Ciencias Sociales, Periodismo e Información</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>Ciencias sociales y del comportamiento</t>
+        </is>
+      </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>Economía</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>Economía</t>
+        </is>
+      </c>
+      <c r="S176" t="inlineStr"/>
+      <c r="T176" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>Humanidades y Cs. Sociales</t>
+        </is>
+      </c>
+      <c r="V176" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>1716</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DE SAN BUENAVENTURA</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Valle del Cauca</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Santiago de Cali</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>107747</v>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>PROFESIONAL EN DANZA Y PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>144</v>
+      </c>
+      <c r="J177" t="n">
+        <v>8</v>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L177" t="n">
+        <v>5189545</v>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N177" s="2" t="n">
+        <v>43558</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>Arte y Humanidades</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>Bellas artes</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>Música</t>
+        </is>
+      </c>
+      <c r="S177" t="inlineStr"/>
+      <c r="T177" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="V177" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>1827</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD CATOLICA DE MANIZALES</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Caldas</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Manizales</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>108754</v>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>ADMINISTRACION DE EMPRESAS TURISTICA</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>156</v>
+      </c>
+      <c r="J178" t="n">
+        <v>10</v>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L178" t="n">
+        <v>5956780</v>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N178" s="2" t="n">
+        <v>43847</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>Gestión y administración</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="S178" t="inlineStr"/>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V178" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-08-18
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V178"/>
+  <dimension ref="A1:V182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17544,10 +17544,8 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>1111</t>
-        </is>
+      <c r="A175" t="n">
+        <v>1111</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -17599,7 +17597,7 @@
           <t>Por cohorte</t>
         </is>
       </c>
-      <c r="N175" s="2" t="n">
+      <c r="N175" s="1" t="n">
         <v>43704</v>
       </c>
       <c r="O175" t="inlineStr">
@@ -17640,10 +17638,8 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>1709</t>
-        </is>
+      <c r="A176" t="n">
+        <v>1709</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -17695,7 +17691,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N176" s="2" t="n">
+      <c r="N176" s="1" t="n">
         <v>45906</v>
       </c>
       <c r="O176" t="inlineStr">
@@ -17736,10 +17732,8 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>1716</t>
-        </is>
+      <c r="A177" t="n">
+        <v>1716</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -17793,7 +17787,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N177" s="2" t="n">
+      <c r="N177" s="1" t="n">
         <v>43558</v>
       </c>
       <c r="O177" t="inlineStr">
@@ -17834,10 +17828,8 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>1827</t>
-        </is>
+      <c r="A178" t="n">
+        <v>1827</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -17891,7 +17883,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N178" s="2" t="n">
+      <c r="N178" s="1" t="n">
         <v>43847</v>
       </c>
       <c r="O178" t="inlineStr">
@@ -17926,6 +17918,396 @@
         </is>
       </c>
       <c r="V178" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>1707</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSIDAD DE BOGOTA - JORGE TADEO LOZANO</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>109144</v>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>CIENCIA DE DATOS Y SIMULACIÓN COMPUTACIONAL</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>125</v>
+      </c>
+      <c r="J179" t="n">
+        <v>8</v>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr"/>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N179" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>Ciencias Naturales, Matemáticas y Estadística</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>Matemáticas y estadística</t>
+        </is>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>Matemáticas, estadística y afines</t>
+        </is>
+      </c>
+      <c r="S179" t="inlineStr"/>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>Ciencias Básicas</t>
+        </is>
+      </c>
+      <c r="V179" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>1710</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD PONTIFICIA BOLIVARIANA</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>108578</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>INGENIERÍA EN CIENCIA DE DATOS</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>144</v>
+      </c>
+      <c r="J180" t="n">
+        <v>9</v>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L180" t="n">
+        <v>12273435</v>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N180" s="2" t="n">
+        <v>43809</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>Tecnologías de la Información y la Comunicación (TIC)</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>Tecnologías de la Información y la Comunicación (TIC)</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>Desarrollo y análisis de software y aplicaciones</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>Ingeniería de sistemas, telemática y afines</t>
+        </is>
+      </c>
+      <c r="S180" t="inlineStr"/>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="V180" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>1714</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>COLEGIO MAYOR DE NUESTRA SEÑORA DEL ROSARIO</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>15613</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>PERIODISMO Y OPINION PUBLICA</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>155</v>
+      </c>
+      <c r="J181" t="n">
+        <v>9</v>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L181" t="n">
+        <v>16667415</v>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N181" s="2" t="n">
+        <v>37326</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>Ciencias Sociales, Periodismo e Información</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>Periodismo e información</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>Periodismo, comunicación y reportajes</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>Comunicación social, periodismo y afines</t>
+        </is>
+      </c>
+      <c r="S181" t="inlineStr"/>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>Humanidades y Cs. Sociales</t>
+        </is>
+      </c>
+      <c r="V181" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>1733</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD SERGIO ARBOLEDA</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Magdalena</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Santa Marta</t>
+        </is>
+      </c>
+      <c r="F182" t="n">
+        <v>5505</v>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>COMUNICACION SOCIAL Y PERIODISMO DIGITAL</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>128</v>
+      </c>
+      <c r="J182" t="n">
+        <v>8</v>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L182" t="n">
+        <v>4799300</v>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N182" s="2" t="n">
+        <v>45119</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>Ciencias Sociales, Periodismo e Información</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>Periodismo e información</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>Periodismo, comunicación y reportajes</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>Comunicación social, periodismo y afines</t>
+        </is>
+      </c>
+      <c r="S182" t="inlineStr"/>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>Humanidades y Cs. Sociales</t>
+        </is>
+      </c>
+      <c r="V182" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-08-25
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V182"/>
+  <dimension ref="A1:V183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17924,10 +17924,8 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>1707</t>
-        </is>
+      <c r="A179" t="n">
+        <v>1707</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -17979,7 +17977,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N179" s="2" t="n">
+      <c r="N179" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="O179" t="inlineStr">
@@ -18020,10 +18018,8 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>1710</t>
-        </is>
+      <c r="A180" t="n">
+        <v>1710</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -18077,7 +18073,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N180" s="2" t="n">
+      <c r="N180" s="1" t="n">
         <v>43809</v>
       </c>
       <c r="O180" t="inlineStr">
@@ -18118,10 +18114,8 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>1714</t>
-        </is>
+      <c r="A181" t="n">
+        <v>1714</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -18175,7 +18169,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N181" s="2" t="n">
+      <c r="N181" s="1" t="n">
         <v>37326</v>
       </c>
       <c r="O181" t="inlineStr">
@@ -18216,10 +18210,8 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>1733</t>
-        </is>
+      <c r="A182" t="n">
+        <v>1733</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -18273,7 +18265,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N182" s="2" t="n">
+      <c r="N182" s="1" t="n">
         <v>45119</v>
       </c>
       <c r="O182" t="inlineStr">
@@ -18308,6 +18300,104 @@
         </is>
       </c>
       <c r="V182" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>1813</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DE LOS ANDES</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>104235</v>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>CONTADURÍA INTERNACIONAL</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>144</v>
+      </c>
+      <c r="J183" t="n">
+        <v>9</v>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L183" t="n">
+        <v>26860000</v>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N183" s="2" t="n">
+        <v>42048</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>Contabilidad e impuestos</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>Contaduría pública</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr"/>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-09-01
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V183"/>
+  <dimension ref="A1:V188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18306,10 +18306,8 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>1813</t>
-        </is>
+      <c r="A183" t="n">
+        <v>1813</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -18363,7 +18361,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N183" s="2" t="n">
+      <c r="N183" s="1" t="n">
         <v>42048</v>
       </c>
       <c r="O183" t="inlineStr">
@@ -18398,6 +18396,492 @@
         </is>
       </c>
       <c r="V183" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSITARIA DEL AREA ANDINA</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Cesar</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Valledupar</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>105016</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>ADMINISTRACION DE EMPRESAS</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>158</v>
+      </c>
+      <c r="J184" t="n">
+        <v>9</v>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L184" t="n">
+        <v>4660000</v>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N184" s="2" t="n">
+        <v>42292</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>Gestión y administración</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="S184" t="inlineStr"/>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V184" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSITARIA DEL AREA ANDINA</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>10569</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>CONTADURIA PUBLICA</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>A distancia</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>158</v>
+      </c>
+      <c r="J185" t="n">
+        <v>9</v>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L185" t="n">
+        <v>3205000</v>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N185" s="2" t="n">
+        <v>36754</v>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>Contabilidad e impuestos</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>Contaduría pública</t>
+        </is>
+      </c>
+      <c r="S185" t="inlineStr"/>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V185" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSITARIA DEL AREA ANDINA</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>54359</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>DISEÑO DE MODAS</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>144</v>
+      </c>
+      <c r="J186" t="n">
+        <v>8</v>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N186" s="2" t="n">
+        <v>39840</v>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>Arte y Humanidades</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>Diseño industrial, de moda e interiores</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="S186" t="inlineStr"/>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>Escuela de Arquitectura, Urbanismo y Diseño</t>
+        </is>
+      </c>
+      <c r="V186" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSITARIA DEL AREA ANDINA</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>103230</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>INGENIERÍA DE MINAS</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>170</v>
+      </c>
+      <c r="J187" t="n">
+        <v>10</v>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr"/>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N187" s="2" t="n">
+        <v>41752</v>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>Ingeniería, Industria y Construcción</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>Industria y procesamiento</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>Minería y extracción</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>Ingeniería de minas, metalurgia y afines</t>
+        </is>
+      </c>
+      <c r="S187" t="inlineStr"/>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="V187" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>4702</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>FUNDACION DE EDUCACION SUPERIOR SAN JOSE -FESSANJOSE-</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>105348</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>INGENIERÍA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>158</v>
+      </c>
+      <c r="J188" t="n">
+        <v>9</v>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L188" t="n">
+        <v>4370822</v>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N188" s="2" t="n">
+        <v>42418</v>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>Ingeniería, Industria y Construcción</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>Ingeniería y profesiones afines</t>
+        </is>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>Ingeniería y profesiones afines no clasificadas en otra parte</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>Ingeniería industrial y afines</t>
+        </is>
+      </c>
+      <c r="S188" t="inlineStr"/>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U188" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="V188" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-09-08
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V188"/>
+  <dimension ref="A1:V190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18402,10 +18402,8 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>2728</t>
-        </is>
+      <c r="A184" t="n">
+        <v>2728</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -18459,7 +18457,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N184" s="2" t="n">
+      <c r="N184" s="1" t="n">
         <v>42292</v>
       </c>
       <c r="O184" t="inlineStr">
@@ -18500,10 +18498,8 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>2728</t>
-        </is>
+      <c r="A185" t="n">
+        <v>2728</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -18557,7 +18553,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N185" s="2" t="n">
+      <c r="N185" s="1" t="n">
         <v>36754</v>
       </c>
       <c r="O185" t="inlineStr">
@@ -18598,10 +18594,8 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>2728</t>
-        </is>
+      <c r="A186" t="n">
+        <v>2728</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -18653,7 +18647,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N186" s="2" t="n">
+      <c r="N186" s="1" t="n">
         <v>39840</v>
       </c>
       <c r="O186" t="inlineStr">
@@ -18694,10 +18688,8 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>2728</t>
-        </is>
+      <c r="A187" t="n">
+        <v>2728</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -18749,7 +18741,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N187" s="2" t="n">
+      <c r="N187" s="1" t="n">
         <v>41752</v>
       </c>
       <c r="O187" t="inlineStr">
@@ -18790,10 +18782,8 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>4702</t>
-        </is>
+      <c r="A188" t="n">
+        <v>4702</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -18847,7 +18837,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N188" s="2" t="n">
+      <c r="N188" s="1" t="n">
         <v>42418</v>
       </c>
       <c r="O188" t="inlineStr">
@@ -18882,6 +18872,200 @@
         </is>
       </c>
       <c r="V188" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>1720</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD MARIANA</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Nariño</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Pasto</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>108661</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>LICENCIATURA EN LITERATURA</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>135</v>
+      </c>
+      <c r="J189" t="n">
+        <v>8</v>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr"/>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N189" s="2" t="n">
+        <v>43816</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>Ciencias de la educación</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="S189" t="inlineStr"/>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="U189" t="inlineStr">
+        <is>
+          <t>Instituto de Estudios en Educación</t>
+        </is>
+      </c>
+      <c r="V189" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>3713</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSITARIA PARA EL DESARROLLO HUMANO - UNINPAHU</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>52769</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>COMUNICACION SOCIAL</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>162</v>
+      </c>
+      <c r="J190" t="n">
+        <v>9</v>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L190" t="n">
+        <v>5649375</v>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N190" s="2" t="n">
+        <v>44384</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>Ciencias Sociales, Periodismo e Información</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>Periodismo e información</t>
+        </is>
+      </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>Periodismo, comunicación y reportajes</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>Comunicación social, periodismo y afines</t>
+        </is>
+      </c>
+      <c r="S190" t="inlineStr"/>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>Humanidades y Cs. Sociales</t>
+        </is>
+      </c>
+      <c r="V190" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>